<commit_message>
WIP -  baixar_relatorio_gastos quase completo
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/relatorio_gastos.xlsx
+++ b/src/main/resources/templates/relatorio_gastos.xlsx
@@ -1,20 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathe\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9264"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,9 +18,29 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>RELATÓRIO DE GASTOS</t>
+  </si>
+  <si>
+    <t>DESCRIÇÃO</t>
+  </si>
+  <si>
+    <t>VALOR</t>
+  </si>
+  <si>
+    <t>VENCIMENTO</t>
+  </si>
+  <si>
+    <t>PAGO</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -33,16 +48,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,12 +85,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -328,7 +384,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -336,9 +392,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="18.5546875" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" customWidth="1"/>
+    <col min="4" max="4" width="12.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[STYLE] colocar bordas nas celulas
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/relatorio_gastos.xlsx
+++ b/src/main/resources/templates/relatorio_gastos.xlsx
@@ -33,7 +33,7 @@
     <t>VENCIMENTO</t>
   </si>
   <si>
-    <t>PAGO</t>
+    <t>STATUS</t>
   </si>
 </sst>
 </file>
@@ -106,10 +106,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -384,7 +384,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -402,24 +402,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>